<commit_message>
21 web elements found
</commit_message>
<xml_diff>
--- a/Documentations/Delhivery Site Web Element Locators.xlsx
+++ b/Documentations/Delhivery Site Web Element Locators.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EXPLEO SMARTCLIFF\Documentations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01E09B29-5684-4DC2-BED6-837610047BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C2F106F-8A2E-4290-A93B-0B608B802513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4EAA58EF-A51B-4E61-BD40-D40005479EB9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t>S. No</t>
   </si>
@@ -213,19 +213,78 @@
   <si>
     <t>Live tracking updates &amp; extra support on our App</t>
   </si>
+  <si>
+    <t>div.app-icons div:nth-child(1)</t>
+  </si>
+  <si>
+    <t>//span[text() = "FTL"]</t>
+  </si>
+  <si>
+    <t>FTL</t>
+  </si>
+  <si>
+    <t>div.flex.ml-4 span.leading-normal</t>
+  </si>
+  <si>
+    <t>//div[@class = "faq-header"]</t>
+  </si>
+  <si>
+    <t>Shipment Status</t>
+  </si>
+  <si>
+    <t>div.faq-header</t>
+  </si>
+  <si>
+    <t>Delhivery Image</t>
+  </si>
+  <si>
+    <t>//img[contains(@src , "Delhivery") and @height = "18"]</t>
+  </si>
+  <si>
+    <t>a.nuxt-link-active img[height = "18"]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Need support with your shipment? </t>
+  </si>
+  <si>
+    <t>//div[contains(text() ,"Need support with your shipment?") and contains(@class, "need-support whitespace-nowrap text-right mb-2")]</t>
+  </si>
+  <si>
+    <t>div.need-support.whitespace-nowrap.text-right.mb-2</t>
+  </si>
+  <si>
+    <t>//input[@id = "simple-search"]</t>
+  </si>
+  <si>
+    <t>input#simple-search</t>
+  </si>
+  <si>
+    <t>Input Search Box</t>
+  </si>
+  <si>
+    <t>//div[@class = "faq-question cursor-pointer"]/following-sibling::div/a[1]</t>
+  </si>
+  <si>
+    <t>Download app link</t>
+  </si>
+  <si>
+    <t>div.faq-divider.faq-divider-open div.faq-answer.cursor-auto a#download-app.underline.text-blue-600</t>
+  </si>
+  <si>
+    <t>//input[@name = "phone"]</t>
+  </si>
+  <si>
+    <t>Input for Mobile number</t>
+  </si>
+  <si>
+    <t>input[name = "phone"]</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,9 +366,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -317,13 +376,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -332,7 +385,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -673,45 +733,45 @@
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.28515625" customWidth="1"/>
-    <col min="3" max="3" width="77" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="121.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="92.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -719,16 +779,16 @@
       <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
@@ -916,76 +976,120 @@
       <c r="A17" s="1">
         <v>14</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="6" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="2"/>
+      <c r="D17" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>15</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="B18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>16</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="B19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>56</v>
+      </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>17</v>
       </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="B20" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>18</v>
       </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="B21" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>19</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="B22" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>20</v>
       </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="B23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="E23" s="2"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>21</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="B24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>